<commit_message>
Update debates data - 2026-09-17
</commit_message>
<xml_diff>
--- a/Debats_Jura.xlsx
+++ b/Debats_Jura.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -233,6 +233,28 @@
     <t xml:space="preserve">Sans trop rallonger, je voudrais vous dire que si vous soutenez la minorité Hurni, vous aurez une première solution qui pourra être débattue soit par la commission du Conseil national soit par notre Commission des affaires juridiques, qui pourrait entretemps y réfléchir. Si nous refusons cette proposition de minorité, nous n'aurons rien pour régler ce problème qui est pourtant clair, évident, qui a été soulevé ici et où il y a vraiment une nécessité d'agir. La résolution du problème sera donc reportée aux calendes grecques. Excusez l'expression !
 Donc, je crois qu'il faut prendre ce que l'on a. Comme un bon tiens vaut mieux que deux tu l'auras, je vous invite aujourd'hui, parce qu'il y a un vrai problème, à soutenir ce que vous propose la minorité de la commission, quitte à peut-être améliorer cette solution à un autre moment. Mais au moins, on aura déjà fait un pas dans la bonne direction.
 Il s'agit d'une situation qui est quand même particulière. Comme on l'a dit, c'est dans un avion et pas dans un restaurant, ou sur la route où l'on peut s'arrêter pour faire venir les agents de la force publique. Il y a une question de protection des passagers mais, plus globalement, de sécurité dans l'avion, qu'il faut pouvoir régler. C'est pour cela que, à mon avis, il faut offrir cette protection au personnel qui travaille dans les avions et soutenir la minorité Hurni.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">419593</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Madame Amaudruz, vous évoquez à juste titre l'aspect de cette réforme relatif à l'indemnisation de l'assurance-chômage. Je ne vous ai pas entendu par exemple vous insurger du fait que, pour l'AVS également, les frontaliers sont indemnisés de la même manière que les résidents suisses puisqu'ils ont cotisé en Suisse. Ce combat semble un peu perdu d'avance, parce qu'il n'est pas lié à l'Union européenne, mais à l'OCDE, qui a des principes par rapport à cela. (Remarque intermédiaire du président : A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Madame Amaudruz, vous évoquez à juste titre l'aspect de cette réforme relatif à l'indemnisation de l'assurance-chômage. Je ne vous ai pas entendu par exemple vous insurger du fait que, pour l'AVS également, les frontaliers sont indemnisés de la même manière que les résidents suisses puisqu'ils ont cotisé en Suisse. Ce combat semble un peu perdu d'avance, parce qu'il n'est pas lié à l'Union européenne, mais à l'OCDE, qui a des principes par rapport à cela. (Remarque intermédiaire du président : Avez-vous une question, Monsieur Loïc Dobler ?) Ma question est donc : l'enjeu qui se pose n'est-il pas plutôt l'imposition des frontaliers aussi en Suisse, plutôt que l'indemnisation par le biais du chômage en France ? Ne vous trompez-vous pas de combat avec cette motion ?
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">419672</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nous avons aujourd'hui le plaisir d'accueillir une délégation du canton du Jura et je remercie le président de m'avoir fait l'amitié de la saluer officiellement à la tribune de notre conseil. La délégation est conduite par M. Fabrice Macquat, président du Parlement jurassien, et c'est pour moi, évidemment, une joie et un honneur de pouvoir vous souhaiter la bienvenue dans la salle du Conseil des États. Pour y accéder, vous êtes passés sous la magnifique verrière de la coupole et avez pu admirer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nous avons aujourd'hui le plaisir d'accueillir une délégation du canton du Jura et je remercie le président de m'avoir fait l'amitié de la saluer officiellement à la tribune de notre conseil. La délégation est conduite par M. Fabrice Macquat, président du Parlement jurassien, et c'est pour moi, évidemment, une joie et un honneur de pouvoir vous souhaiter la bienvenue dans la salle du Conseil des États. Pour y accéder, vous êtes passés sous la magnifique verrière de la coupole et avez pu admirer les armoiries des cantons disposées autour de la croix suisse.
+Les guides s'amusent souvent à demander aux visiteuses et visiteurs où se trouvent les armoiries du Jura, car ces dernières ne trônent pas sous la coupole, puisqu'elles ont été ajoutées bien après la construction du Palais du Parlement. Pour cause, son inauguration en 1902 est intervenue 77 ans avant l'entrée en souveraineté du canton. Ainsi, absente de la coupole en 1902, la région jurassienne a néanmoins posé, cette année-là, un jalon important pour rallier un jour la Berne fédérale. Elle a en effet largement approuvé en votation populaire un projet de construction de nouvelle ligne de chemin de fer qui allait préfigurer le percement de la ligne ferroviaire Moutier-Bienne. Lorsqu'en 1979, le canton du Jura est entré en souveraineté au terme d'une histoire que l'on sait mouvementée, ces armoiries ont trouvé une place de choix au-dessus des trois Confédérés.
+La Confédération que nous représentons aujourd'hui n'est pas celle qui s'est unie sous cette coupole en 1902. Elle a changé, elle s'est agrandie, elle a évolué avec les générations et les territoires qui la composent. Unies sous un même toit, les armoiries sous la coupole sont le témoin de cette histoire. Elles nous rappellent, à l'instar du canton du Jura, que le fédéralisme sur lequel la Suisse s'est construite depuis ses origines porte les graines des changements dont la population se fait le moteur. Je vous souhaite une très cordiale bienvenue au Palais fédéral ainsi qu'une excellente visite. (Applaudissements)
 </t>
   </si>
 </sst>
@@ -287,8 +309,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I11" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I13" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I13"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -905,6 +927,64 @@
         <v>52</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>53</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" t="s">
+        <v>23</v>
+      </c>
+      <c r="H12" t="s">
+        <v>54</v>
+      </c>
+      <c r="I12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" t="s">
+        <v>23</v>
+      </c>
+      <c r="H13" t="s">
+        <v>57</v>
+      </c>
+      <c r="I13" t="s">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-09-29
</commit_message>
<xml_diff>
--- a/Debats_Jura.xlsx
+++ b/Debats_Jura.xlsx
@@ -504,7 +504,7 @@
   <si>
     <t xml:space="preserve">Ce postulat s'inscrit pleinement dans notre politique des agglomérations transfrontalières, dont l'importance est aujourd'hui d'autant plus soulignée par la votation du canton de Genève sur le financement des P+R de l'autre côté de la frontière. Nos agglomérations transfrontalières, qu'il s'agisse de Genève, Bâle, Lugano ou du Chablais, sont les moteurs de notre économie. Mais aujourd'hui, le coût de cette activité est un engorgement quotidien de nos réseaux routiers. Chaque matin, ce sont des colonnes ininterrompues de véhicules individuels qui traversent nos communes.
 Selon l'Office fédéral de la statistique (OFS), plus de 80 pour cent de la totalité des frontaliers actifs en Suisse travaillent dans des cantons limitrophes de la France comme Genève, Vaud, Neuchâtel et le Jura, et au Tessin. En 2021, la grande majorité d'entre eux utilisaient la voiture individuelle pour leurs déplacements quotidiens, représentant le coeur du trafic aux frontières. L'Office fédéral des routes (OFROU) recense plus de 68 000 heures d'embouteillage sur nos autoroutes, ce qui provoque un report massif du trafic sur nos routes secondaires. L'Office fédéral du développement territorial (ARE) évalue les coûts externes totaux de la mobilité individuelle en Suisse à près de 10 milliards de francs par an. Les habitantes et habitants de nos communes frontalières, de nos agglomérations, en payent directement le prix : bruit permanent, dégradation de l'air, risque pour la sécurité routière, usure permanente des routes locales - à la charge des communes - et péjoration de la qualité de vie.
-Dans son avis, le Conseil fédéral nous dit que tout va bien, que les instruments actuels comme l'OPTA ou la loi sur les chemins de fer suffisent et que le principe de territorialité doit prévaloir. Il nous rappelle les 850 millions de francs investis par le passé dans des projets emblématiques comme le CEVA ou Mendrisio-Varese.
+Dans son avis, le Conseil fédéral nous dit que tout va bien, que les instruments actuels comme l'Ordonnance du DETEC concernant le programme en faveur du trafic d'agglomération (OPTA) ou la loi sur les chemins de fer suffisent et que le principe de territorialité doit prévaloir. Il nous rappelle les 850 millions de francs investis par le passé dans des projets emblématiques comme le CEVA ou Mendrisio-Varese.
 Mais cela n'est pas suffisant pour garantir un développement territorial harmonieux et cohérent. Face à cela, les solutions concrètes existent pourtant et passent par un report modal efficace : créer et renforcer des lignes de transports publics transfrontalières - bus à haute fréquence, trams, liaisons ferroviaires ou lignes express. Lorsque nous offrons une alternative rapide et directe de l'autre côté de la frontière, nous stoppons les voitures avant qu'elles ne viennent s'engorger dans nos villages. Regardez l'exemple du Léman Express et ses plus de 80 000 voyageurs par jour. La preuve est faite : dès qu'une alternative crédible existe, le report modal fonctionne.
 Avec ce postulat, je demande d'adapter nos outils financiers pour accélérer ces mesures de transports publics ciblées et rendre aux usagères et usagers de la route la fluidité dont ils ont besoin. Pour le bien-être, le bien-vivre ensemble dans nos communes et le dynamisme de nos régions frontalières, je vous invite donc à soutenir ce postulat.
 </t>
@@ -571,15 +571,15 @@
 Les arguments politiques ne manquent pas et les arguments économiques en faveur de ces textes sont indiscutables.
 Tout d'abord, le poids massif de l'UE dans notre commerce. L'Union européenne reste de très loin notre principal partenaire commercial. Cela a été dit : plus de 50 pour cent des exportations de marchandises suisses, soit plus de 147 milliards de francs par an, sont destinés au marché européen. En sens inverse, environ 70 pour cent de nos importations en proviennent.
 Ensuite, il y a un impact direct sur l'emploi suisse. Notre économie dépend de conditions-cadres fiables. En moyenne, une entreprise suisse sur deux emploie de la main-d'oeuvre qualifiée issue de l'UE. Bloquer ce paquet, c'est mettre en péril la compétitivité de nos entreprises et la sécurité de milliers d'emplois helvétiques.
-Ces chiffres sont impressionnants à l'échelle nationale. Ils deviennent une question de survie économique pour les cantons de l'Arc jurassien. Je veux parler des cantons de Neuchâtel, du Jura, de la région du Jura bernois et du Nord vaudois, qui sont des régions frontalières. Une économie ultra exportatrice, l'Arc jurassien, abrite les fleurons de l'horlogerie, des microtechniques, des machines et des technologies médicales. C'est une région dont la richesse repose presque exclusivement sur sa capacité à exporter. Deux francs sur trois sont gagnés à l'étranger. 
-Sans la mise à jour des accords, notamment sur la suppression des obstacles techniques au commerce, l'industrie de l'Arc jurassien fera face à des barrières administratives majeures qui détruiront sa compétitivité face à la concurrence mondiale. Voilà un exemple qui était souhaité par notre collègue Salzmann. Ce n'est pas une projection, mais nous l'avons vécu récemment. 
-La réalité transfrontalière : l'Arc jurassien vit et respire au rythme de la coopération transfrontalière. Près de 72 000 frontaliers - 12 000 pour le seul canton du Jura - viennent chaque jour y apporter leurs compétences essentielles. Stabiliser la libre circulation des personnes et sécuriser l'accès au marché du travail est une condition sine qua non pour que le tissu industriel de l'Arc jurassien puisse continuer à produire et à innover. 
-Étant donné qu'on a parlé des effets du Brexit - on a parlé de l'évolution de son PIB -, j'ai profité de ce long débat pour vérifier sur les réseaux, respectivement au travers de l'intelligence artificielle, quelle était la situation. Les chiffres sont clairs. Le PIB du Royaume-Uni a progressé moins vite que celui de l'Union européenne, entre 6 et 8 pour cent. Quant à la productivité de ce pays, il a baissé de 3 pour cent et l'emploi a baissé de 4 pour cent à cause des frictions administratives et des coûts des échanges depuis le Brexit. 
-Quant à l'aspect institutionnel, qui a souvent monopolisé le débat au détriment du contenu des accords, il serait regrettable, comme l'a dit notre collègue Chassot, que ce soit l'arbre qui cache la forêt. Nous y reviendrons, mais je vous invite déjà à appliquer la Constitution que nous avons promis de respecter au début de notre mandat. Elle règle complètement la question des compétences et notamment de l'application du référendum facultatif. Pourquoi faudrait-il la triturer et la torturer pour lui faire dire autre chose que ce qu'elle contient ? 
+Ces chiffres sont impressionnants à l'échelle nationale. Ils deviennent une question de survie économique pour les cantons de l'Arc jurassien. Je veux parler des cantons de Neuchâtel, du Jura, de la région du Jura bernois et du Nord vaudois, qui sont des régions frontalières avec une économie ultra exportatrice. L'Arc jurassien abrite les fleurons de l'horlogerie, des microtechniques, des machines et des technologies médicales. C'est une région dont la richesse repose presque exclusivement sur sa capacité à exporter. Deux francs sur trois sont gagnés à l'étranger.
+Sans la mise à jour des accords, notamment sur la suppression des obstacles techniques au commerce, l'industrie de l'Arc jurassien fera face à des barrières administratives majeures qui détruiront sa compétitivité face à la concurrence mondiale. Voilà un exemple, comme l'avait souhaité notre collègue Salzmann. Ce n'est pas une projection ; nous l'avons vécu récemment.
+La réalité transfrontalière : l'Arc jurassien vit et respire au rythme de la coopération transfrontalière. Près de 72 000 frontaliers - 12 000 pour le seul canton du Jura - viennent chaque jour y apporter leurs compétences essentielles. Stabiliser la libre circulation des personnes et sécuriser l'accès au marché du travail est une condition sine qua non pour que le tissu industriel de l'Arc jurassien puisse continuer à produire et à innover.
+Étant donné qu'on a parlé des effets du Brexit - on a parlé de l'évolution du PIB -, j'ai profité de ce long débat pour vérifier sur les réseaux, respectivement au travers de l'intelligence artificielle, quelle était la situation. Les chiffres sont clairs. Le PIB du Royaume-Uni a progressé moins vite que celui de l'Union européenne, entre 6 et 8 pour cent. Quant à la productivité de ce pays, elle a diminué de 3 pour cent et l'emploi a baissé de 4 pour cent à cause des frictions administratives et des coûts des échanges depuis le Brexit.
+Quant à l'aspect institutionnel, qui a souvent monopolisé le débat au détriment du contenu des accords, il serait regrettable, comme l'a dit notre collègue Chassot, que ce soit l'arbre qui cache la forêt. Nous y reviendrons, mais je vous invite déjà à appliquer la Constitution que nous avons promis de respecter au début de notre mandat. Elle règle complètement la question des compétences et notamment de l'application du référendum facultatif. Pourquoi faudrait-il la triturer et la torturer pour lui faire dire autre chose que ce qu'elle contient ?
 Vous l'aurez compris : à l'instar des cantons romands, je soutiens le référendum facultatif. Ces cantons estiment en effet avoir été suffisamment associés aux préparations des actes législatifs dont nous allons parler et que leurs remarques et demandes ont été suffisamment prises en compte par le Conseil fédéral.
 Il est d'ailleurs curieux d'entendre les tenants de la souveraineté de notre pays citer à l'envi des professeurs étrangers et ignorer les avis de la quasi-totalité des professeurs de droit constitutionnel de notre pays.
-En conclusion, les cantons de Suisse occidentale, les entreprises et les associations professionnelles sont unis pour réclamer cette sécurité juridique indispensable à la bonne marge de leurs affaires. L'isolement n'est pas une option viable, il en va de la prospérité de notre pays et, par voie de conséquence, du pouvoir d'achat et du bien-être de nos concitoyennes et concitoyens. Nous avons besoin de coconstruire ensemble la voie bilatérale qui a largement contribué à la prospérité et la souveraineté de notre pays.
-Je vous invite à entrer en matière sur ce projet, à mener un débat constructif tourné vers l'avenir et finalement à accepter les projets qui nous sont soumis.
+En conclusion, les cantons de Suisse occidentale, les entreprises et les associations professionnelles sont unis pour réclamer cette sécurité juridique indispensable à la bonne marche de leurs affaires. L'isolement n'est pas une option viable. Il en va de la prospérité de notre pays et, par voie de conséquence, du pouvoir d'achat et du bien-être de nos concitoyennes et concitoyens. Nous avons besoin de coconstruire ensemble la voie bilatérale, qui a largement contribué à la prospérité et la souveraineté de notre pays.
+Je vous invite à entrer en matière sur ce projet, à mener un débat constructif tourné vers l'avenir et, finalement, à accepter les projets qui nous sont soumis.
 </t>
   </si>
   <si>
@@ -587,25 +587,25 @@
   </si>
   <si>
     <t xml:space="preserve">Dans la mode, on classifie les habits entre S et XL. Aujourd'hui, on a aussi inventé le XXL. Le débat d'aujourd'hui, c'est un débat XXL. Je ne vais pas répéter ce qui a été dit, mais je vais quand même apporter quelques arguments qui concernent mon canton, puisque l'on a beaucoup entendu ce jour la voix des cantons.
-Tout d'abord, pourquoi un débat XXL ? Des auditions publiques - c'est quasiment une première -, 32 séances de commissions, des plénières importantes, des commissions avec chaque fois</t>
+Tout d'abord, pourquoi un débat XXL ? Des auditions publiques - c'est quasiment une première -, 32 séances de commissions, des séances plénières importantes, des commissions avec cha</t>
   </si>
   <si>
     <t xml:space="preserve">Dans la mode, on classifie les habits entre S et XL. Aujourd'hui, on a aussi inventé le XXL. Le débat d'aujourd'hui, c'est un débat XXL. Je ne vais pas répéter ce qui a été dit, mais je vais quand même apporter quelques arguments qui concernent mon canton, puisque l'on a beaucoup entendu ce jour la voix des cantons.
-Tout d'abord, pourquoi un débat XXL ? Des auditions publiques - c'est quasiment une première -, 32 séances de commissions, des plénières importantes, des commissions avec chaque fois des leaders, trois conseillers fédéraux présents - c'est très rare de voir une délégation aussi importante devant notre chambre -, la présence de la presse - c'est rare aussi de voir les tribunes de la presse si fournies. Cela veut dire que c'est un débat qui est important. Certains ont qualifié le débat comme "la mère de toutes les batailles". À titre personnel, ce n'est pas la mère de toutes les batailles. C'est un dossier parmi d'autres. Mais c'est un dossier qui est important.
-Nous sommes responsables de notre vote. Nous sommes 46. Notre vote correspond également à notre diversité cantonale. À vous entendre, certains considèrent que l'Europe est un ennemi. Non, l'Europe, c'est un partenaire économique, de fait, les chiffres ont été rappelés. De temps en temps, nous sommes en concurrence avec l'Europe. Nos industries, de temps en temps, sont en concurrence avec l'Europe. Et notre devoir, c'est de trouver un chemin pour que notre économie puisse prospérer, se développer et créer de la richesse qui est utile à la cohésion sociale.
-J'ai entendu ce mot qui devient de plus en plus magique : la souveraineté. La souveraineté peut être unique quand vous êtes sur une île, mais quand vous êtes au milieu de l'Europe, la souveraineté, c'est aussi trouver des partenariats qui consolident le pays. Certes, c'est un mot magique pour nous, les Suisses, mais en même temps, la souveraineté se partage, que ce soit dans le domaine militaire, de la sécurité ou de l'approvisionnement. D'ailleurs, on vient d'avoir une votation le week-end dernier sur la souveraineté alimentaire. Et on constate que, dans tous les cas de figure, il n'y aura pas de souveraineté alimentaire au niveau suisse. Même durant le plan Wahlen, il n'y a pas eu de souveraineté alimentaire au niveau suisse. Nous devons compter également avec d'autres pays. Nous devons construire des stratégies avec d'autres pays.
-Ensuite, j'en suis très heureux, quand on donne la parole au peuple, le peuple s'exprime. Notre chambre a longuement débattu de l'initiative populaire "Pas de Suisse à 10 millions ! (initiative pour la durabilité)". Pour certains, il fallait faire un contre-projet ; pour d'autres, et j'étais de ceux-là, un contre-projet, non, mais par contre, affronter le peuple, expliquer que quand nous avons une pyramide des âges avec un vieillissement majeur, nous avons intérêt à trouver des solutions pour garantir un équilibre de la pyramide des âges, garantir les emplois. Je rappelle que dans le cadre du débat que nous avons eu concernant l'initiative "Pas de Suisse à 10 millions ! (initiative pour la durabilité)", nous avons mis en place des garde-fous. La Suisse, en permanence, peut se fermer ou se réouvrir. Ce qui a été négocié par le Conseil fédéral permet d'avoir une clause de sauvegarde ; en tout temps, on peut la dénoncer. Non pas comme l'ont fait les Anglais avec le Brexit, mais dénoncer une clause. 
-Ensuite, la neutralité. Là aussi, nous avons eu un débat très large, intense. 75 pour cent du peuple suisse a dit non à l'initiative populaire "Sauvegarder la neutralité suisse (initiative sur la neutralité)", et j'en suis très heureux. 
-Flexibilité, stabilité, prévisibilité, sécurité juridique : c'est cela que nous amène ce dossier qui a été négocié par le Conseil fédéral. Stabilité, pour continuer à travailler par la voie bilatérale. Prévisibilité, pour nos entreprises : un entrepreneur a besoin de savoir, en lien avec son cahier de commandes, ce qu'il va se passer ces prochaines années. Et sécurité juridique : quand il y a un accord, il y a deux parties. Il y a des arbitres qui traiteront de l'accord. Cela permet d'avoir une sécurité juridique dans un monde en pleine évolution. 
-Cela me fait beaucoup sourire : il y a quelques mois - et là je remercie le président de la Confédération, M. Parmelin, qui essaie de travailler sur les taxes américaines -, on pensait que l'Europe, c'était l'ennemi, et qu'on avait trouvé des marchés assez simples. Les États-Unis sont devenus un marché, mais les règles ont beaucoup changé avec nos amis américains. Nous aurons à débattre, et suivant le chemin que nous choisirons dans le domaine des accords internationaux, avec le Mercosur, je me réjouis déjà qu'il faille avoir une double majorité concernant l'accord avec le Mercosur. Je me réjouis déjà. 
-Un autre dossier qui va venir prochainement, c'est celui de la Chine. Il n'y a pas un jour où l'on ne lit pas que, demain, la Chine sera la plus grande puissance économique mondiale. Je me réjouis d'avoir un débat, et si une nouvelle fois, nous devons soumettre ce texte à une double majorité, cela sera compliqué, parce que la Chine est loin, elle n'est pas si proche de notre marché. Notre marché, c'est l'Europe, l'Europe des 27.
-Ce que je n'ai pas beaucoup entendu dans le débat d'aujourd'hui c'est des remerciements. Je pense que c'est important de savoir remercier les gens qui ont fait un travail très important. J'ai présidé à la destinée des 26 cantons avec mon collègue Würth, au sein de cette chambre. On a commencé le débat sur les Bilatérales `III il y a à peu près 15 ans. Le conseiller fédéral Burkhalter a travaillé sur ce dossier, a mis en place le dialogue Europe. Il a quitté le Conseil fédéral, et le conseiller fédéral Cassis, vice-président du Conseil fédéral, a repris le flambeau. Il y a bientôt dix ans qu'il travaille sur ce dossier, et ce n'est pas simple. Personnellement, je souhaitais vous remercier, Messieurs, pour l'engagement que vous avez manifesté pour la Suisse. Tous les jours, c'était un dossier sensible, complexe, avec votre administration et les ambassadeurs, vous avez trouvé un chemin qui est utile à la cohésion de ce pays.
+Tout d'abord, pourquoi un débat XXL ? Des auditions publiques - c'est quasiment une première -, 32 séances de commissions, des séances plénières importantes, des commissions avec chaque fois des leaders, trois conseillers fédéraux présents - c'est très rare de voir une délégation aussi importante devant notre chambre -, la présence de la presse - c'est rare aussi de voir les tribunes de la presse si fournies. Cela veut dire que c'est un débat qui est important. Certains ont qualifié le débat comme étant "la mère de toutes les batailles". À titre personnel, ce n'est pas la mère de toutes les batailles. C'est un dossier parmi d'autres, mais c'est un dossier qui est important.
+Nous sommes responsables de notre vote. Nous sommes 46. Notre vote correspond également à notre diversité cantonale. À vous entendre, certains considèrent que l'Europe est un ennemi. Non, l'Europe, c'est un partenaire économique, les chiffres ont été rappelés. De temps en temps, nous sommes en concurrence avec l'Europe. Nos industries, de temps en temps, sont en concurrence avec l'Europe. Notre devoir est de trouver un chemin pour que notre économie puisse prospérer, se développer et créer de la richesse qui est utile à la cohésion sociale.
+J'ai entendu ce mot qui devient de plus en plus magique : la souveraineté. La souveraineté peut être unique quand vous êtes sur une île, mais quand vous êtes au milieu de l'Europe, la souveraineté, c'est aussi trouver des partenariats qui consolident le pays. Certes, c'est un mot magique pour nous, les Suisses, mais en même temps, la souveraineté se partage, que ce soit dans le domaine militaire, de la sécurité ou de l'approvisionnement. D'ailleurs, on vient d'avoir une votation le week-end dernier sur la souveraineté alimentaire. On constate que, dans tous les cas de figure, il n'y aura pas de souveraineté alimentaire au niveau suisse. Même durant le plan Wahlen, il n'y a pas eu de souveraineté alimentaire au niveau suisse. Nous devons compter également avec d'autres pays. Nous devons construire des stratégies avec d'autres pays.
+Ensuite, j'en suis très heureux, quand on donne la parole au peuple, le peuple s'exprime. Notre chambre a longuement débattu de l'initiative populaire "Pas de Suisse à 10 millions ! (initiative pour la durabilité)". Pour certains, il fallait faire un contre-projet ; pour d'autres - et j'étais de ceux-là - pas de contre-projet, mais par contre, il fallait affronter le peuple et expliquer que quand nous avons une pyramide des âges avec un vieillissement majeur, nous avons intérêt à trouver des solutions pour garantir un équilibre de la pyramide des âges et garantir les emplois. Je rappelle que dans le cadre du débat que nous avons eu concernant l'initiative "Pas de Suisse à 10 millions ! (initiative pour la durabilité)", nous avons mis en place des garde-fous. La Suisse peut en permanence se fermer ou se réouvrir. Ce qui a été négocié par le Conseil fédéral permet d'avoir une clause de sauvegarde ; en tout temps, on peut la dénoncer - non pas comme l'ont fait les Anglais avec le Brexit, mais dénoncer une clause.
+Ensuite, la neutralité. Là aussi, nous avons eu un débat très large et intense. 75 pour cent du peuple suisse a dit non à l'initiative populaire "Sauvegarder la neutralité suisse (initiative sur la neutralité)", et j'en suis très heureux.
+Flexibilité, stabilité, prévisibilité, sécurité juridique : c'est cela que nous amène ce dossier qui a été négocié par le Conseil fédéral. Stabilité, pour continuer à travailler par la voie bilatérale. Prévisibilité, pour nos entreprises : un entrepreneur a besoin de savoir, en lien avec son cahier de commandes, ce qu'il va se passer ces prochaines années. Et sécurité juridique : quand il y a un accord, il y a deux parties, mais il y a aussi des arbitres qui traiteront de l'accord, et cela permet d'avoir une sécurité juridique dans un monde en pleine évolution.
+Cela me fait beaucoup sourire : il y a quelques mois - et là, je remercie le président de la Confédération, M. Parmelin, qui essaie de travailler sur les taxes américaines -, on pensait que l'Europe était l'ennemi, et qu'on allait trouver des marchés assez simplement. Les États-Unis sont devenus un marché, mais les règles ont beaucoup changé avec nos amis américains. Nous aurons à débattre, suivant le chemin que nous choisirons dans le domaine des accords internationaux, du Mercosur. Je me réjouis déjà qu'il faille avoir une double majorité concernant l'accord avec le Mercosur - je me réjouis déjà.
+Un autre dossier qui va venir prochainement, c'est celui de la Chine. Il n'y a pas un jour où l'on ne lit pas que, demain, la Chine sera la plus grande puissance économique mondiale. Je me réjouis d'avoir un débat. Si une nouvelle fois, nous devons soumettre ce texte à une double majorité, cela sera compliqué, parce que la Chine est loin, elle n'est pas si proche de notre marché. Notre marché, c'est l'Europe : l'Europe des 27.
+Ce que je n'ai pas beaucoup entendu dans le débat d'aujourd'hui,ce sont des remerciements. Je pense que c'est important de savoir remercier les gens qui ont fait un travail très important. J'ai présidé à la destinée des 26 cantons avec mon collègue Würth, au sein de cette chambre. On a commencé le débat sur les Bilatérales III il y a à peu près 15 ans. Le conseiller fédéral Burkhalter a travaillé sur ce dossier, a mis en place le dialogue Europe. Il a quitté le Conseil fédéral et le conseiller fédéral Cassis, vice-président du Conseil fédéral, a repris le flambeau. Il y a bientôt dix ans qu'il travaille sur ce dossier et ce n'est pas simple. Personnellement, je souhaitais vous remercier, Messieurs, pour l'engagement que vous avez manifesté pour la Suisse, tous les jours. C'était un dossier sensible, complexe. Avec votre administration et les ambassadeurs, vous avez trouvé un chemin qui est utile à la cohésion de ce pays.
 J'aimerais également remercier les cantons. J'ai entendu aujourd'hui la voix des cantons. Chaque canton, c'est la force de notre pays, qui est plurielle. Quand on est à Schwytz, on n'est pas à Lausanne, c'est clair. Et quand on est à Lausanne, on n'est pas dans le Jura ni en Valais ou dans le canton d'Uri. Chaque canton a ses spécificités. En vous écoutant, j'ai entendu que vous avez amené aujourd'hui, dans le cadre de ce débat, ces spécificités régionales. Ce que je sais, c'est que quand nous sommes unis, nous créons la Suisse. Et la Suisse crée de la richesse, de la cohésion, de l'ouverture et de l'intelligence.
-Le débat que nous avons aujourd'hui - et c'est pour cela que je vous encourage à entrer en matière -, c'est un débat important, qui permettra d'avoir de la prospective, et créer justement cette Suisse qu'on aime.
-J'aimerais remercier également les partenaires sociaux. Parce que pour moi, l'Europe, c'est avant tout économique, puisqu'on contrôle notre marché du travail. Les partenaires sociaux dans ce dossier ont travaillé - c'était difficile, je le sais : notre collègue Maillard a travaillé, au nom de l'USS, avec d'autres partenaires. La partie adverse, l'économie, a trouvé un chemin : 14 mesures, que je soutiendrai, car je pense qu'elles s'inscrivent dans une logique très claire. Il s'agit de garantir le pouvoir d'achat, les salaires, la cohésion et de nouveau, la stabilité et les équilibres, la prévisibilité. C'est dans cet esprit que j'ai compris ce dossier.
-Je ne souhaitais pas intervenir, mais comme chaque canton s'est exprimé en apportant son éclairage, je vais parler encore quelques minutes de mon canton de Vaud. C'est le troisième canton suisse, bientôt à un million d'habitants, et j'en suis très fier. Cela ne me pose aucun problème que nous ayons un million d'habitants, parce que nous avons une pyramide des âges équilibrée, entre les personnes qui vieillissent, les jeunes qui doivent trouver une destinée et ceux qui sont dans le monde du travail.
- Ensuite, nous avons les hautes écoles. Nous traiterons tout à l'heure ou demain d'Erasmus plus. Là aussi il faut de la prévisibilité. Quand nous n'avons pas signé les accords avec le milieu académique et autres, on a pleuré et il a fallu trouver des solutions. On doit stabiliser ce dossier pour le bien de nos enfants. On n'a pas de pétrole, mais par contre on a des hautes écoles et nos hautes écoles doivent avoir des partenariats équilibrés avec l'étranger. Là aussi il en va de la sécurité.
-Dernier point concernant mon canton, c'est un canton ouvert qui, lors des votations, a des positions parmi les plus ouvertes au niveau suisse. L'ouverture, c'est tout le contraire de la fermeture. Quand un canton se ferme, quand un pays se ferme, pendant quelques années, il peut peut-être vivre sur cette notion de souveraineté, quoique aujourd'hui on est dépendant des uns des autres, on le voit avec les taxes américaines. C'est pour ça que le canton de Vaud a dit à la députation vaudoise dans cette chambre de soutenir le travail du Conseil fédéral que nous remercions sincèrement pour avoir atteint les objectifs et pour le projet qui est sur la table. Je vous encourage à en faire de même, à entrer en matière, à améliorer si on peut le faire deux ou trois points de l'accord général puis à l'envoyer au Conseil national pour qu'il puisse l'examiner et ainsi trouver une destinée pour notre pays, de la stabilité, de la prévisibilité et de la sécurité juridique dans un monde en pleine évolution et insécuritaire.
+Le débat que nous avons aujourd'hui - et c'est pour cela que je vous encourage à entrer en matière -, c'est un débat important, qui permettra d'avoir de la perspective et de créer justement cette Suisse qu'on aime.
+J'aimerais remercier également les partenaires sociaux. Parce que pour moi, l'Europe, c'est avant tout économique, puisqu'on contrôle notre marché du travail. Les partenaires sociaux dans ce dossier ont travaillé - c'était difficile, je le sais : notre collègue Maillard a travaillé, au nom de l'Union syndicale suisse (USS), avec d'autres partenaires. La partie adverse, l'économie, a trouvé un chemin : 14 mesures, que je soutiendrai, car je pense qu'elles s'inscrivent dans une logique très claire. Il s'agit de garantir le pouvoir d'achat, les salaires, la cohésion et, de nouveau, la stabilité et les équilibres, la prévisibilité. C'est dans cet esprit que j'ai compris ce dossier.
+Je ne souhaitais pas intervenir, mais comme chaque canton s'est exprimé en apportant son éclairage, je vais parler encore quelques minutes de mon canton de Vaud. C'est le troisième canton suisse. Bientôt un million d'habitants et j'en suis très fier. Cela ne me pose aucun problème que nous ayons un million d'habitants, parce que nous avons une pyramide des âges équilibrée, entre les personnes qui vieillissent, les jeunes qui doivent trouver une destinée et ceux qui sont dans le monde du travail.
+Ensuite, nous avons les hautes écoles. Nous traiterons tout à l'heure ou demain d'Erasmus plus. Là aussi il faut de la prévisibilité. Quand nous n'avons pas signé les accords avec le milieu académique et autres, on a pleuré et il a fallu trouver des solutions. On doit stabiliser ce dossier pour le bien de nos enfants. On n'a pas de pétrole, mais par contre on a de hautes écoles et nos hautes écoles doivent avoir des partenariats équilibrés avec l'étranger. Là aussi il en va de la sécurité.
+Dernier point concernant mon canton, c'est un canton ouvert qui, lors des votations, a des positions parmi les plus ouvertes sur le plan suisse. L'ouverture, c'est tout le contraire de la fermeture. Quand un canton se ferme, quand un pays se ferme, pendant quelques années, il peut peut-être vivre sur cette notion de souveraineté, quoiqu'aujourd'hui on soit dépendant les uns des autres, on le voit avec les taxes américaines. C'est pour cela que le canton de Vaud a dit à la députation vaudoise dans cette chambre de soutenir le travail du Conseil fédéral que nous remercions sincèrement pour avoir atteint les objectifs et pour le projet qui est sur la table. Je vous encourage à en faire de même, à entrer en matière, à améliorer, si on peut le faire, deux ou trois points de l'accord général puis à l'envoyer au Conseil national pour qu'il puisse l'examiner et ainsi trouver une destinée pour notre pays, de la stabilité, de la prévisibilité et de la sécurité juridique dans un monde en pleine évolution et insécuritaire.
 </t>
   </si>
   <si>
@@ -634,13 +634,15 @@
 Wir müssen sorgfältig abwägen, was wir heute tun. Es ist der wichtigste strategische Entscheid unseres Landes für die nächsten Jahrzehnte, ja, für die nächsten Generationen. Wir sollten nicht zaudern. Die Verträge geben uns das Instrumentarium für eine selbstbewusste Umsetzung, die unseren Interessen Rechnung trägt. Diesen Spielraum müssen wir selbstbewusst nutzen. Ich bin davon überzeugt, dass wir das tun und mit unseren Beratungen auch zeigen werden.
 Die Antwort - Sie merken es - ist daher für mich klar: Eintreten auf das Stabilisierungspaket mit der EU und Ja zur Weiterentwicklung unserer heute schon erfolgreichen Beziehungen, statt noch mehr zu verzögern. Und Ja zum fakultativen Staatsvertragsreferendum, damit die betroffenen Stimmbürgerinnen und Stimmbürger allein entscheiden können, denn sie sind direkt betroffen - sie und ihre Nachkommen.
 Die Schweiz ist nicht trotz ihrer Verflechtung mit Europa erfolgreich. Sie ist vor allem aufgrund ihrer Verbundenheit mit Europa erfolgreich. Die Schweiz ist Europa - eigentlich komisch, dass man das immer wiederholen muss. Jetzt geht es darum, diese Verbindungen für die Zukunft zu sichern. Die Welt um uns herum ist nämlich unsicherer geworden. Gerade in solchen Zeiten wäre es töricht, die Beziehungen zu unseren wichtigsten und verlässlichsten Partnern unnötig zu schwächen.
-Der internationale Handel wird härter. Macht gilt vor Recht. Wollen Sie mit solchen Staaten weitere Verträge abschliessen, Freihandelsabkommen, und Staatsverträge aushandeln, und übermorgen ist wieder alles anders? Wir haben Herausforderungen mit der zukünftigen Energieversorgung. Fragen der Forschung, Gesundheit und Sicherheit müssen wir bewältigen, und nicht nur die Schweiz steht vor diesen Herausforderungen. Wir haben mit diesem Extremsommer einen Fingerzeig der Klimakrise erlebt. Das können wir als Schweiz nicht alleine lösen, mitten in Europa. Wir sollten das gemeinsam tun. Deshalb ist es wichtig, dass wir diese Weiterentwicklung unserer Beziehungen zur EU als unserem stabilsten Partner weiterverfolgen.
-Die Herren Schmid und Stark sagten vorhin, es könnten ja einfach die Bilateralen I und II weitergeführt werden. Das ist Selbstbetrug, geschätzte Kollegen, es tut mir leid. Denn wir wissen heute, und das können Ihnen alle bestätigen, und die Wirtschaft spürt bereits, dass das nicht stimmt. Unsere heutigen Abkommen erodieren, weil es in den 25 Jahren in der EU, in der Welt und auch in der Schweiz so viele Veränderungen gegeben hat. Stellen Sie sich vor, wie schnell sich alles verändert! Wir sind weder im Jahr 1291, die geschätzte Kollegin Z'graggen ist noch nicht da, und wir sind auch nicht im Jahre 2000, geschätzter Kollege Schmid.
-Ich gebe ein Beispiel. Unsere Pharma- und Medtech-Firmen sowie die Maschinenindustrie sind ganz direkt und unmittelbar betroffen, wenn die gegenseitige Anerkennung der technischen Standards nicht mehr aktualisiert wird. Zahlreiche Konzerne und KMU mit Sitz in der Nordwestschweiz sind auf einen diskriminierungsfreien Zugang zum europäischen Markt angewiesen. Ohne die Bilateralen werden Firmen ihre Investitionen eher im Ausland tätigen. Soll ich Ihnen sagen, was das Ausland bedeutet? Es bedeutet einfach: fünf Kilometer verschieben, über die Landesgrenze ins Elsass oder nach Südbaden oder in andere Regionen. 15 Kantone in unserem Land sind Grenzregionen. Das heisst, es ist eigentlich einfach. Dies hat direkte Auswirkungen auf Arbeitsplätze und die Volkswirtschaft, und auf unser Wissen. Wissen ist nämlich die wichtigste Ressource der Schweiz, und es definiert unsere Zukunft, besonders für den Innovations- und Life-Science-Standort Nordwestschweiz. Wissen braucht Vernetzung, weswegen der Zugang zu den EU-Programmen Horizon Europe und Erasmus plus für den Forschungsplatz Schweiz unverzichtbar ist.
-Noch ein Wort als Vertreterin der Nordwestschweiz und des Kantons Basel-Landschaft: In der Nordwestschweizer Regierungskonferenz sind die Kantone Solothurn, Aargau, Basel-Stadt, Jura und Basel-Landschaft vertreten. Sie haben gemeinsam bekräftigt, dass geregelte Beziehungen zur Europäischen Union unverzichtbar sind. Sie sind überzeugt, dass das Verhandlungsergebnis geregelte Beziehungen mit der EU ermöglicht und den bilateralen Weg absichert und weiterentwickelt. Sie wissen als Grenzregionen, wie eng verflochten die Beziehungen zu den benachbarten EU-Staaten sind. Sie sind für die Nordwestschweizer Kantone existenziell. Ich möchte hier auch noch darauf hinweisen, dass es darum geht, dass daher auch offene Grenzen in Verbindung mit der Absicherung des Schweizer Lohnschutzniveaus elementar für einen funktionierenden Arbeitsmarkt, gute wirtschaftliche Zusammenarbeit und den gesellschaftlichen Zusammenhalt in einer Grenzregion sind.
-Diese klare Haltung kommt nicht von ungefähr. Die Nordwestschweiz ist die exportstärkste Region der Schweiz. Fast die Hälfte aller Schweizer Exporte kommen aus der Nordwestschweiz, wovon wiederum die Hälfte in die EU als wichtigsten Handelspartner der Schweiz geht. Das kann niemand von heute auf morgen einfach ersetzen. Es ist nicht ersetzbar. Das sind unsere Nachbarn, die wichtigsten Handelspartner.
-Ich bin überzeugt, dass wir eine Schweiz wollen, die ihre Zukunft selbstbewusst gestaltet, keine Schweiz, die aus Angst vor Veränderungen Schritt für Schritt sich selbst ins Abseits stellt und sich auch noch ideologisch verschanzt. Die Bilateralen III sind kein Abschied von unserer nationalen Entscheidungsfreiheit. Wir werden hier als Parlament immer entscheiden und immer auch das letzte Wort haben. Das ist wichtig und muss gewährleistet sein, und das ist es auch. Die Bilateralen III sind die Fortsetzung eines Weges, den die Schweiz vor 25 Jahren eingeschlagen hat: eigenständig bleiben und trotzdem eng mit unseren europäischen Nachbarn zusammenarbeiten. Genau das wird mit dem Paket bezweckt, das nun vorliegt. 
-Ich will diese souveräne Schweiz, eine Schweiz, die ihren Kindern nicht nur Wohlstand hinterlässt, sondern eben auch gesunde Lebensgrundlagen und eine vielfältige Gesellschaft sowie Freiheit, Demokratie und Rechtsstaatlichkeit. Das können wir gemeinsam erreichen. Daran müssen wir gemeinsam arbeiten. Ich will eine Schweiz, die weiterhin mitredet und mitbestimmt, und zwar dort, wo sie ihre Zukunft beeinflussen kann. Ich will keine Schweiz, die nur reagiert und immer hinterherspringt und sich dann beugen muss, wenn Macht vor Recht gilt. Daher ist für mich klar: Ich trete ein und werde auch mit Überzeugung diesem EU-Vertragspaket zustimmen.
+Der internationale Handel wird zunehmend härter. Macht gilt vor Recht. Wollen Sie mit solchen Staaten weitere Verträge, Freihandelsabkommen abschliessen und Staatsverträge aushandeln - und übermorgen ist wieder alles anders?
+Wir haben Herausforderungen mit der zukünftigen Energieversorgung, wir müssen Fragen der Forschung, Gesundheit und Sicherheit bewältigen, und vor diesen Herausforderungen steht nicht nur die Schweiz. Dieser Extremsommer war ein Fingerzeig der Klimakrise. Das alles können wir als Schweiz mitten in Europa nicht alleine lösen. Wir sollten das gemeinsam tun. Deshalb ist es wichtig, dass wir diese Weiterentwicklung unserer Beziehungen zur EU als unserem stabilsten Partner weiterverfolgen.
+Die Herren Schmid und Stark sagten vorhin, es könnten ja einfach die Bilateralen I und II weitergeführt werden. Das ist Selbstbetrug, geschätzte Kollegen, es tut mir leid. Wir wissen - das können Ihnen alle bestätigen und die Wirtschaft spürt es bereits -, dass das nicht stimmt. Unsere heutigen Abkommen erodieren, weil es in den letzten 25 Jahren in der EU, in der Welt und auch in der Schweiz sehr viele Veränderungen gegeben hat. Denken Sie daran, wie schnell sich alles verändert. Wir sind weder im Jahr 1291, geschätzte Kollegin Z'graggen, noch sind wir im Jahr 2000, geschätzter Kollege Schmid.
+Ich gebe ein Beispiel. Unsere Pharma- und Medtech-Firmen sowie die Maschinenindustrie sind ganz direkt und unmittelbar betroffen, wenn die gegenseitige Anerkennung der technischen Standards nicht mehr aktualisiert wird. Zahlreiche Konzerne und KMU mit Sitz in der Nordwestschweiz sind auf einen diskriminierungsfreien Zugang zum europäischen Markt angewiesen. Ohne die Bilateralen werden Firmen ihre Investitionen eher im Ausland tätigen. Soll ich Ihnen sagen, was das Ausland bedeutet? Es bedeutet einfach: fünf Kilometer verschieben, über die Landesgrenze ins Elsass oder nach Südbaden oder in andere Regionen. 15 Kantone in unserem Land sind Grenzregionen. Das heisst, es ist eigentlich einfach, es hat direkte Auswirkungen auf Arbeitsplätze und die Volkswirtschaft - und auf unser Wissen. Wissen ist nämlich die wichtigste Ressource der Schweiz, und es definiert unsere Zukunft, besonders für den Innovations- und Life-Science-Standort Nordwestschweiz. Wissen braucht Vernetzung, weswegen der Zugang zu den EU-Programmen Horizon Europe und Erasmus plus für den Forschungsplatz Schweiz unverzichtbar ist.
+Noch ein Wort als Vertreterin der Nordwestschweiz und des Kantons Basel-Landschaft: In der Nordwestschweizer Regierungskonferenz sind die Kantone Solothurn, Aargau, Basel-Stadt, Jura und Basel-Landschaft vertreten. Sie haben gemeinsam bekräftigt, dass geregelte Beziehungen zur Europäischen Union unverzichtbar sind. Sie sind überzeugt, dass das Verhandlungsergebnis geregelte Beziehungen mit der EU ermöglicht und den bilateralen Weg absichert und weiterentwickelt. Sie wissen als Grenzregionen, wie eng verflochten die Beziehungen zu den benachbarten EU-Staaten sind. Sie sind für die Nordwestschweizer Kantone existenziell. Ich möchte auch noch darauf hinweisen, dass offene Grenzen in Verbindung mit der Absicherung des Schweizer Lohnschutzniveaus elementar für einen funktionierenden Arbeitsmarkt, gute wirtschaftliche Zusammenarbeit und den gesellschaftlichen Zusammenhalt in einer Grenzregion sind.
+Diese klare Haltung kommt nicht von ungefähr. Die Nordwestschweiz ist die exportstärkste Region der Schweiz. Fast die Hälfte aller Schweizer Exporte kommt aus der Nordwestschweiz, wovon wiederum die Hälfte in die EU als wichtigsten Handelspartner der Schweiz geht. Das kann niemand von heute auf morgen einfach ersetzen. Es ist nicht ersetzbar. Das sind unsere Nachbarn, die wichtigsten Handelspartner.
+Ich bin überzeugt, dass wir eine Schweiz wollen, die ihre Zukunft selbstbewusst gestaltet, keine Schweiz, die aus Angst vor Veränderungen sich Schritt für Schritt selbst ins Abseits stellt und sich auch noch ideologisch verschanzt. Die Bilateralen III sind kein Abschied von unserer nationalen Entscheidungsfreiheit. Wir werden hier als Parlament immer entscheiden und immer auch das letzte Wort haben. Das ist wichtig und muss gewährleistet sein, und das ist es auch. Die Bilateralen III sind die Fortsetzung eines Weges, den die Schweiz vor 25 Jahren eingeschlagen hat: eigenständig bleiben und trotzdem eng mit unseren europäischen Nachbarn zusammenarbeiten. Genau das wird mit dem Paket bezweckt, das nun vorliegt. 
+Ich will diese souveräne Schweiz, eine Schweiz, die ihren Kindern nicht nur Wohlstand hinterlässt, sondern eben auch gesunde Lebensgrundlagen und eine vielfältige Gesellschaft sowie Freiheit, Demokratie und Rechtsstaatlichkeit. Das können wir gemeinsam erreichen. Daran müssen wir gemeinsam arbeiten. Ich will eine Schweiz, die weiterhin mitredet und mitbestimmt, und zwar dort, wo sie ihre Zukunft beeinflussen kann. Ich will keine Schweiz, die nur reagiert und immer hinterherspringt und sich dann beugen muss, wenn Macht vor Recht gilt.
+Daher ist für mich klar: Ich trete ein und werde diesem EU-Vertragspaket auch mit Überzeugung zustimmen.
 </t>
   </si>
 </sst>

</xml_diff>